<commit_message>
Update parliament data - 2026-03-03
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3633" uniqueCount="3633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="3634">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -10185,9 +10185,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-03</t>
-  </si>
-  <si>
     <t xml:space="preserve">Staatspolitik|Medien und Kommunikation|Menschenrechte</t>
   </si>
   <si>
@@ -10224,6 +10221,9 @@
     <t xml:space="preserve">25.4562</t>
   </si>
   <si>
+    <t xml:space="preserve">Le Centre</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unbürokratische Entlastung bei invasiven Schadorganismen</t>
   </si>
   <si>
@@ -10294,6 +10294,9 @@
   </si>
   <si>
     <t xml:space="preserve">25.4614</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PS</t>
   </si>
   <si>
     <t xml:space="preserve">Medikamente als Kostentreiber in der obligatorischen Krankenpflegeversicherung?</t>
@@ -31224,17 +31227,15 @@
         <v>35</v>
       </c>
       <c r="R305"/>
-      <c r="S305" t="s">
+      <c r="S305"/>
+      <c r="T305" t="s">
         <v>3390</v>
       </c>
-      <c r="T305" t="s">
+      <c r="U305" t="s">
         <v>3391</v>
       </c>
-      <c r="U305" t="s">
+      <c r="V305" t="s">
         <v>3392</v>
-      </c>
-      <c r="V305" t="s">
-        <v>3393</v>
       </c>
     </row>
     <row r="306">
@@ -31242,7 +31243,7 @@
         <v>20254696</v>
       </c>
       <c r="B306" t="s">
-        <v>3394</v>
+        <v>3393</v>
       </c>
       <c r="C306" t="s">
         <v>40</v>
@@ -31263,28 +31264,28 @@
         <v>563</v>
       </c>
       <c r="I306" t="s">
+        <v>3394</v>
+      </c>
+      <c r="J306" t="s">
         <v>3395</v>
       </c>
-      <c r="J306" t="s">
+      <c r="K306" t="s">
         <v>3396</v>
       </c>
-      <c r="K306" t="s">
+      <c r="L306" t="s">
         <v>3397</v>
       </c>
-      <c r="L306" t="s">
+      <c r="M306" t="s">
         <v>3398</v>
-      </c>
-      <c r="M306" t="s">
-        <v>3399</v>
       </c>
       <c r="N306" t="s">
         <v>50</v>
       </c>
       <c r="O306" t="s">
+        <v>3399</v>
+      </c>
+      <c r="P306" t="s">
         <v>3400</v>
-      </c>
-      <c r="P306" t="s">
-        <v>3401</v>
       </c>
       <c r="Q306" t="s">
         <v>89</v>
@@ -31306,7 +31307,7 @@
         <v>20254562</v>
       </c>
       <c r="B307" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="C307" t="s">
         <v>232</v>
@@ -31315,7 +31316,7 @@
         <v>1568</v>
       </c>
       <c r="E307" t="s">
-        <v>79</v>
+        <v>3402</v>
       </c>
       <c r="F307" t="s">
         <v>43</v>
@@ -31379,7 +31380,7 @@
         <v>3414</v>
       </c>
       <c r="E308" t="s">
-        <v>79</v>
+        <v>3402</v>
       </c>
       <c r="F308" t="s">
         <v>43</v>
@@ -31443,7 +31444,7 @@
         <v>2013</v>
       </c>
       <c r="E309" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F309" t="s">
         <v>43</v>
@@ -31455,28 +31456,28 @@
         <v>97</v>
       </c>
       <c r="I309" t="s">
-        <v>3427</v>
+        <v>3428</v>
       </c>
       <c r="J309" t="s">
-        <v>3428</v>
+        <v>3429</v>
       </c>
       <c r="K309" t="s">
-        <v>3429</v>
+        <v>3430</v>
       </c>
       <c r="L309" t="s">
-        <v>3430</v>
+        <v>3431</v>
       </c>
       <c r="M309" t="s">
-        <v>3431</v>
+        <v>3432</v>
       </c>
       <c r="N309" t="s">
         <v>50</v>
       </c>
       <c r="O309" t="s">
-        <v>3432</v>
+        <v>3433</v>
       </c>
       <c r="P309" t="s">
-        <v>3433</v>
+        <v>3434</v>
       </c>
       <c r="Q309" t="s">
         <v>53</v>
@@ -31498,19 +31499,19 @@
         <v>20258194</v>
       </c>
       <c r="B310" t="s">
-        <v>3434</v>
+        <v>3435</v>
       </c>
       <c r="C310" t="s">
         <v>59</v>
       </c>
       <c r="D310" t="s">
-        <v>3435</v>
+        <v>3436</v>
       </c>
       <c r="E310" t="s">
         <v>61</v>
       </c>
       <c r="F310" t="s">
-        <v>3436</v>
+        <v>3437</v>
       </c>
       <c r="G310" t="s">
         <v>27</v>
@@ -31519,26 +31520,26 @@
         <v>97</v>
       </c>
       <c r="I310" t="s">
-        <v>3437</v>
+        <v>3438</v>
       </c>
       <c r="J310" t="s">
-        <v>3438</v>
+        <v>3439</v>
       </c>
       <c r="K310"/>
       <c r="L310" t="s">
-        <v>3439</v>
+        <v>3440</v>
       </c>
       <c r="M310" t="s">
-        <v>3440</v>
+        <v>3441</v>
       </c>
       <c r="N310" t="s">
         <v>69</v>
       </c>
       <c r="O310" t="s">
-        <v>3441</v>
+        <v>3442</v>
       </c>
       <c r="P310" t="s">
-        <v>3442</v>
+        <v>3443</v>
       </c>
       <c r="Q310" t="s">
         <v>53</v>
@@ -31560,7 +31561,7 @@
         <v>20258273</v>
       </c>
       <c r="B311" t="s">
-        <v>3443</v>
+        <v>3444</v>
       </c>
       <c r="C311" t="s">
         <v>59</v>
@@ -31572,7 +31573,7 @@
         <v>659</v>
       </c>
       <c r="F311" t="s">
-        <v>3436</v>
+        <v>3437</v>
       </c>
       <c r="G311" t="s">
         <v>27</v>
@@ -31581,26 +31582,26 @@
         <v>97</v>
       </c>
       <c r="I311" t="s">
-        <v>3444</v>
+        <v>3445</v>
       </c>
       <c r="J311" t="s">
-        <v>3445</v>
+        <v>3446</v>
       </c>
       <c r="K311"/>
       <c r="L311" t="s">
-        <v>3446</v>
+        <v>3447</v>
       </c>
       <c r="M311" t="s">
-        <v>3447</v>
+        <v>3448</v>
       </c>
       <c r="N311" t="s">
         <v>69</v>
       </c>
       <c r="O311" t="s">
-        <v>3448</v>
+        <v>3449</v>
       </c>
       <c r="P311" t="s">
-        <v>3449</v>
+        <v>3450</v>
       </c>
       <c r="Q311" t="s">
         <v>89</v>
@@ -31608,13 +31609,13 @@
       <c r="R311"/>
       <c r="S311"/>
       <c r="T311" t="s">
-        <v>3450</v>
+        <v>3451</v>
       </c>
       <c r="U311" t="s">
-        <v>3451</v>
+        <v>3452</v>
       </c>
       <c r="V311" t="s">
-        <v>3452</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="312">
@@ -31622,7 +31623,7 @@
         <v>20254463</v>
       </c>
       <c r="B312" t="s">
-        <v>3453</v>
+        <v>3454</v>
       </c>
       <c r="C312" t="s">
         <v>77</v>
@@ -31634,7 +31635,7 @@
         <v>659</v>
       </c>
       <c r="F312" t="s">
-        <v>3454</v>
+        <v>3455</v>
       </c>
       <c r="G312" t="s">
         <v>27</v>
@@ -31643,28 +31644,28 @@
         <v>63</v>
       </c>
       <c r="I312" t="s">
-        <v>3455</v>
+        <v>3456</v>
       </c>
       <c r="J312" t="s">
-        <v>3456</v>
+        <v>3457</v>
       </c>
       <c r="K312" t="s">
-        <v>3457</v>
+        <v>3458</v>
       </c>
       <c r="L312" t="s">
-        <v>3458</v>
+        <v>3459</v>
       </c>
       <c r="M312" t="s">
-        <v>3459</v>
+        <v>3460</v>
       </c>
       <c r="N312" t="s">
         <v>69</v>
       </c>
       <c r="O312" t="s">
-        <v>3460</v>
+        <v>3461</v>
       </c>
       <c r="P312" t="s">
-        <v>3461</v>
+        <v>3462</v>
       </c>
       <c r="Q312" t="s">
         <v>35</v>
@@ -31686,19 +31687,19 @@
         <v>20254281</v>
       </c>
       <c r="B313" t="s">
-        <v>3462</v>
+        <v>3463</v>
       </c>
       <c r="C313" t="s">
         <v>232</v>
       </c>
       <c r="D313" t="s">
-        <v>3463</v>
+        <v>3464</v>
       </c>
       <c r="E313" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F313" t="s">
-        <v>3464</v>
+        <v>3465</v>
       </c>
       <c r="G313" t="s">
         <v>27</v>
@@ -31707,28 +31708,28 @@
         <v>563</v>
       </c>
       <c r="I313" t="s">
-        <v>3465</v>
+        <v>3466</v>
       </c>
       <c r="J313" t="s">
-        <v>3466</v>
+        <v>3467</v>
       </c>
       <c r="K313" t="s">
-        <v>3467</v>
+        <v>3468</v>
       </c>
       <c r="L313" t="s">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="M313" t="s">
-        <v>3469</v>
+        <v>3470</v>
       </c>
       <c r="N313" t="s">
         <v>50</v>
       </c>
       <c r="O313" t="s">
-        <v>3470</v>
+        <v>3471</v>
       </c>
       <c r="P313" t="s">
-        <v>3471</v>
+        <v>3472</v>
       </c>
       <c r="Q313" t="s">
         <v>89</v>
@@ -31750,7 +31751,7 @@
         <v>20254317</v>
       </c>
       <c r="B314" t="s">
-        <v>3472</v>
+        <v>3473</v>
       </c>
       <c r="C314" t="s">
         <v>77</v>
@@ -31762,7 +31763,7 @@
         <v>42</v>
       </c>
       <c r="F314" t="s">
-        <v>3464</v>
+        <v>3465</v>
       </c>
       <c r="G314" t="s">
         <v>27</v>
@@ -31771,28 +31772,28 @@
         <v>563</v>
       </c>
       <c r="I314" t="s">
-        <v>3473</v>
+        <v>3474</v>
       </c>
       <c r="J314" t="s">
-        <v>3474</v>
+        <v>3475</v>
       </c>
       <c r="K314" t="s">
-        <v>3475</v>
+        <v>3476</v>
       </c>
       <c r="L314" t="s">
-        <v>3476</v>
+        <v>3477</v>
       </c>
       <c r="M314" t="s">
-        <v>3477</v>
+        <v>3478</v>
       </c>
       <c r="N314" t="s">
         <v>50</v>
       </c>
       <c r="O314" t="s">
-        <v>3478</v>
+        <v>3479</v>
       </c>
       <c r="P314" t="s">
-        <v>3479</v>
+        <v>3480</v>
       </c>
       <c r="Q314" t="s">
         <v>89</v>
@@ -31800,13 +31801,13 @@
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>3480</v>
+        <v>3481</v>
       </c>
       <c r="U314" t="s">
-        <v>3481</v>
+        <v>3482</v>
       </c>
       <c r="V314" t="s">
-        <v>3482</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="315">
@@ -31814,19 +31815,19 @@
         <v>20254145</v>
       </c>
       <c r="B315" t="s">
-        <v>3483</v>
+        <v>3484</v>
       </c>
       <c r="C315" t="s">
         <v>77</v>
       </c>
       <c r="D315" t="s">
-        <v>3484</v>
+        <v>3485</v>
       </c>
       <c r="E315" t="s">
         <v>42</v>
       </c>
       <c r="F315" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G315" t="s">
         <v>81</v>
@@ -31835,28 +31836,28 @@
         <v>63</v>
       </c>
       <c r="I315" t="s">
-        <v>3486</v>
+        <v>3487</v>
       </c>
       <c r="J315" t="s">
-        <v>3487</v>
+        <v>3488</v>
       </c>
       <c r="K315" t="s">
-        <v>3488</v>
+        <v>3489</v>
       </c>
       <c r="L315" t="s">
-        <v>3489</v>
+        <v>3490</v>
       </c>
       <c r="M315" t="s">
-        <v>3490</v>
+        <v>3491</v>
       </c>
       <c r="N315" t="s">
         <v>69</v>
       </c>
       <c r="O315" t="s">
-        <v>3491</v>
+        <v>3492</v>
       </c>
       <c r="P315" t="s">
-        <v>3492</v>
+        <v>3493</v>
       </c>
       <c r="Q315" t="s">
         <v>53</v>
@@ -31878,19 +31879,19 @@
         <v>20254188</v>
       </c>
       <c r="B316" t="s">
-        <v>3493</v>
+        <v>3494</v>
       </c>
       <c r="C316" t="s">
         <v>77</v>
       </c>
       <c r="D316" t="s">
-        <v>3494</v>
+        <v>3495</v>
       </c>
       <c r="E316" t="s">
         <v>42</v>
       </c>
       <c r="F316" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G316" t="s">
         <v>81</v>
@@ -31899,28 +31900,28 @@
         <v>97</v>
       </c>
       <c r="I316" t="s">
-        <v>3495</v>
+        <v>3496</v>
       </c>
       <c r="J316" t="s">
-        <v>3496</v>
+        <v>3497</v>
       </c>
       <c r="K316" t="s">
-        <v>3497</v>
+        <v>3498</v>
       </c>
       <c r="L316" t="s">
-        <v>3498</v>
+        <v>3499</v>
       </c>
       <c r="M316" t="s">
-        <v>3499</v>
+        <v>3500</v>
       </c>
       <c r="N316" t="s">
         <v>3387</v>
       </c>
       <c r="O316" t="s">
-        <v>3500</v>
+        <v>3501</v>
       </c>
       <c r="P316" t="s">
-        <v>3501</v>
+        <v>3502</v>
       </c>
       <c r="Q316" t="s">
         <v>53</v>
@@ -31942,7 +31943,7 @@
         <v>20254225</v>
       </c>
       <c r="B317" t="s">
-        <v>3502</v>
+        <v>3503</v>
       </c>
       <c r="C317" t="s">
         <v>40</v>
@@ -31954,7 +31955,7 @@
         <v>659</v>
       </c>
       <c r="F317" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G317" t="s">
         <v>27</v>
@@ -31963,28 +31964,28 @@
         <v>97</v>
       </c>
       <c r="I317" t="s">
-        <v>3503</v>
+        <v>3504</v>
       </c>
       <c r="J317" t="s">
-        <v>3504</v>
+        <v>3505</v>
       </c>
       <c r="K317" t="s">
-        <v>3505</v>
+        <v>3506</v>
       </c>
       <c r="L317" t="s">
-        <v>3506</v>
+        <v>3507</v>
       </c>
       <c r="M317" t="s">
-        <v>3507</v>
+        <v>3508</v>
       </c>
       <c r="N317" t="s">
         <v>50</v>
       </c>
       <c r="O317" t="s">
-        <v>3508</v>
+        <v>3509</v>
       </c>
       <c r="P317" t="s">
-        <v>3509</v>
+        <v>3510</v>
       </c>
       <c r="Q317" t="s">
         <v>89</v>
@@ -31992,13 +31993,13 @@
       <c r="R317"/>
       <c r="S317"/>
       <c r="T317" t="s">
-        <v>3510</v>
+        <v>3511</v>
       </c>
       <c r="U317" t="s">
-        <v>3511</v>
+        <v>3512</v>
       </c>
       <c r="V317" t="s">
-        <v>3512</v>
+        <v>3513</v>
       </c>
     </row>
     <row r="318">
@@ -32006,19 +32007,19 @@
         <v>20254234</v>
       </c>
       <c r="B318" t="s">
-        <v>3513</v>
+        <v>3514</v>
       </c>
       <c r="C318" t="s">
         <v>77</v>
       </c>
       <c r="D318" t="s">
-        <v>3514</v>
+        <v>3515</v>
       </c>
       <c r="E318" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F318" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G318" t="s">
         <v>27</v>
@@ -32027,28 +32028,28 @@
         <v>97</v>
       </c>
       <c r="I318" t="s">
-        <v>3515</v>
+        <v>3516</v>
       </c>
       <c r="J318" t="s">
-        <v>3516</v>
+        <v>3517</v>
       </c>
       <c r="K318" t="s">
-        <v>3517</v>
+        <v>3518</v>
       </c>
       <c r="L318" t="s">
-        <v>3518</v>
+        <v>3519</v>
       </c>
       <c r="M318" t="s">
-        <v>3519</v>
+        <v>3520</v>
       </c>
       <c r="N318" t="s">
         <v>69</v>
       </c>
       <c r="O318" t="s">
-        <v>3520</v>
+        <v>3521</v>
       </c>
       <c r="P318" t="s">
-        <v>3521</v>
+        <v>3522</v>
       </c>
       <c r="Q318" t="s">
         <v>35</v>
@@ -32056,13 +32057,13 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>3522</v>
+        <v>3523</v>
       </c>
       <c r="U318" t="s">
-        <v>3523</v>
+        <v>3524</v>
       </c>
       <c r="V318" t="s">
-        <v>3524</v>
+        <v>3525</v>
       </c>
     </row>
     <row r="319">
@@ -32070,19 +32071,19 @@
         <v>20254071</v>
       </c>
       <c r="B319" t="s">
-        <v>3525</v>
+        <v>3526</v>
       </c>
       <c r="C319" t="s">
         <v>40</v>
       </c>
       <c r="D319" t="s">
-        <v>3526</v>
+        <v>3527</v>
       </c>
       <c r="E319" t="s">
         <v>42</v>
       </c>
       <c r="F319" t="s">
-        <v>3527</v>
+        <v>3528</v>
       </c>
       <c r="G319" t="s">
         <v>81</v>
@@ -32091,28 +32092,28 @@
         <v>97</v>
       </c>
       <c r="I319" t="s">
-        <v>3528</v>
+        <v>3529</v>
       </c>
       <c r="J319" t="s">
-        <v>3529</v>
+        <v>3530</v>
       </c>
       <c r="K319" t="s">
-        <v>3530</v>
+        <v>3531</v>
       </c>
       <c r="L319" t="s">
-        <v>3531</v>
+        <v>3532</v>
       </c>
       <c r="M319" t="s">
-        <v>3532</v>
+        <v>3533</v>
       </c>
       <c r="N319" t="s">
         <v>69</v>
       </c>
       <c r="O319" t="s">
-        <v>3533</v>
+        <v>3534</v>
       </c>
       <c r="P319" t="s">
-        <v>3534</v>
+        <v>3535</v>
       </c>
       <c r="Q319" t="s">
         <v>53</v>
@@ -32120,13 +32121,13 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>3535</v>
+        <v>3536</v>
       </c>
       <c r="U319" t="s">
-        <v>3536</v>
+        <v>3537</v>
       </c>
       <c r="V319" t="s">
-        <v>3537</v>
+        <v>3538</v>
       </c>
     </row>
     <row r="320">
@@ -32134,7 +32135,7 @@
         <v>20254024</v>
       </c>
       <c r="B320" t="s">
-        <v>3538</v>
+        <v>3539</v>
       </c>
       <c r="C320" t="s">
         <v>40</v>
@@ -32143,10 +32144,10 @@
         <v>1639</v>
       </c>
       <c r="E320" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F320" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G320" t="s">
         <v>27</v>
@@ -32155,28 +32156,28 @@
         <v>44</v>
       </c>
       <c r="I320" t="s">
-        <v>3540</v>
+        <v>3541</v>
       </c>
       <c r="J320" t="s">
-        <v>3541</v>
+        <v>3542</v>
       </c>
       <c r="K320" t="s">
-        <v>3542</v>
+        <v>3543</v>
       </c>
       <c r="L320" t="s">
-        <v>3543</v>
+        <v>3544</v>
       </c>
       <c r="M320" t="s">
-        <v>3544</v>
+        <v>3545</v>
       </c>
       <c r="N320" t="s">
         <v>50</v>
       </c>
       <c r="O320" t="s">
-        <v>3545</v>
+        <v>3546</v>
       </c>
       <c r="P320" t="s">
-        <v>3546</v>
+        <v>3547</v>
       </c>
       <c r="Q320" t="s">
         <v>89</v>
@@ -32198,7 +32199,7 @@
         <v>20257863</v>
       </c>
       <c r="B321" t="s">
-        <v>3547</v>
+        <v>3548</v>
       </c>
       <c r="C321" t="s">
         <v>59</v>
@@ -32210,7 +32211,7 @@
         <v>1848</v>
       </c>
       <c r="F321" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G321" t="s">
         <v>27</v>
@@ -32219,26 +32220,26 @@
         <v>63</v>
       </c>
       <c r="I321" t="s">
-        <v>3548</v>
+        <v>3549</v>
       </c>
       <c r="J321" t="s">
-        <v>3549</v>
+        <v>3550</v>
       </c>
       <c r="K321"/>
       <c r="L321" t="s">
-        <v>3550</v>
+        <v>3551</v>
       </c>
       <c r="M321" t="s">
-        <v>3551</v>
+        <v>3552</v>
       </c>
       <c r="N321" t="s">
         <v>69</v>
       </c>
       <c r="O321" t="s">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="P321" t="s">
-        <v>3553</v>
+        <v>3554</v>
       </c>
       <c r="Q321" t="s">
         <v>53</v>
@@ -32260,7 +32261,7 @@
         <v>20257888</v>
       </c>
       <c r="B322" t="s">
-        <v>3554</v>
+        <v>3555</v>
       </c>
       <c r="C322" t="s">
         <v>59</v>
@@ -32269,10 +32270,10 @@
         <v>1495</v>
       </c>
       <c r="E322" t="s">
-        <v>1496</v>
+        <v>659</v>
       </c>
       <c r="F322" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G322" t="s">
         <v>27</v>
@@ -32281,26 +32282,26 @@
         <v>44</v>
       </c>
       <c r="I322" t="s">
-        <v>3555</v>
+        <v>3556</v>
       </c>
       <c r="J322" t="s">
-        <v>3556</v>
+        <v>3557</v>
       </c>
       <c r="K322"/>
       <c r="L322" t="s">
-        <v>3557</v>
+        <v>3558</v>
       </c>
       <c r="M322" t="s">
-        <v>3558</v>
+        <v>3559</v>
       </c>
       <c r="N322" t="s">
         <v>69</v>
       </c>
       <c r="O322" t="s">
-        <v>3559</v>
+        <v>3560</v>
       </c>
       <c r="P322" t="s">
-        <v>3560</v>
+        <v>3561</v>
       </c>
       <c r="Q322" t="s">
         <v>35</v>
@@ -32322,7 +32323,7 @@
         <v>20257890</v>
       </c>
       <c r="B323" t="s">
-        <v>3561</v>
+        <v>3562</v>
       </c>
       <c r="C323" t="s">
         <v>59</v>
@@ -32334,7 +32335,7 @@
         <v>659</v>
       </c>
       <c r="F323" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G323" t="s">
         <v>27</v>
@@ -32343,26 +32344,26 @@
         <v>563</v>
       </c>
       <c r="I323" t="s">
-        <v>3562</v>
+        <v>3563</v>
       </c>
       <c r="J323" t="s">
-        <v>3563</v>
+        <v>3564</v>
       </c>
       <c r="K323"/>
       <c r="L323" t="s">
-        <v>3564</v>
+        <v>3565</v>
       </c>
       <c r="M323" t="s">
-        <v>3565</v>
+        <v>3566</v>
       </c>
       <c r="N323" t="s">
         <v>69</v>
       </c>
       <c r="O323" t="s">
-        <v>3566</v>
+        <v>3567</v>
       </c>
       <c r="P323" t="s">
-        <v>3567</v>
+        <v>3568</v>
       </c>
       <c r="Q323" t="s">
         <v>89</v>
@@ -32384,17 +32385,17 @@
         <v>20254003</v>
       </c>
       <c r="B324" t="s">
-        <v>3568</v>
+        <v>3569</v>
       </c>
       <c r="C324" t="s">
         <v>232</v>
       </c>
       <c r="D324" t="s">
-        <v>3569</v>
+        <v>3570</v>
       </c>
       <c r="E324"/>
       <c r="F324" t="s">
-        <v>3570</v>
+        <v>3571</v>
       </c>
       <c r="G324" t="s">
         <v>27</v>
@@ -32403,28 +32404,28 @@
         <v>63</v>
       </c>
       <c r="I324" t="s">
-        <v>3571</v>
+        <v>3572</v>
       </c>
       <c r="J324" t="s">
-        <v>3572</v>
+        <v>3573</v>
       </c>
       <c r="K324" t="s">
-        <v>3573</v>
+        <v>3574</v>
       </c>
       <c r="L324" t="s">
-        <v>3574</v>
+        <v>3575</v>
       </c>
       <c r="M324" t="s">
-        <v>3575</v>
+        <v>3576</v>
       </c>
       <c r="N324" t="s">
         <v>50</v>
       </c>
       <c r="O324" t="s">
-        <v>3576</v>
+        <v>3577</v>
       </c>
       <c r="P324" t="s">
-        <v>3577</v>
+        <v>3578</v>
       </c>
       <c r="Q324" t="s">
         <v>53</v>
@@ -32432,13 +32433,13 @@
       <c r="R324"/>
       <c r="S324"/>
       <c r="T324" t="s">
-        <v>3578</v>
+        <v>3579</v>
       </c>
       <c r="U324" t="s">
-        <v>3579</v>
+        <v>3580</v>
       </c>
       <c r="V324" t="s">
-        <v>3580</v>
+        <v>3581</v>
       </c>
     </row>
     <row r="325">
@@ -32446,7 +32447,7 @@
         <v>20253984</v>
       </c>
       <c r="B325" t="s">
-        <v>3581</v>
+        <v>3582</v>
       </c>
       <c r="C325" t="s">
         <v>77</v>
@@ -32456,7 +32457,7 @@
       </c>
       <c r="E325"/>
       <c r="F325" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G325" t="s">
         <v>27</v>
@@ -32465,28 +32466,28 @@
         <v>63</v>
       </c>
       <c r="I325" t="s">
-        <v>3486</v>
+        <v>3487</v>
       </c>
       <c r="J325" t="s">
-        <v>3487</v>
+        <v>3488</v>
       </c>
       <c r="K325" t="s">
-        <v>3488</v>
+        <v>3489</v>
       </c>
       <c r="L325" t="s">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="M325" t="s">
-        <v>3584</v>
+        <v>3585</v>
       </c>
       <c r="N325" t="s">
         <v>3420</v>
       </c>
       <c r="O325" t="s">
-        <v>3585</v>
+        <v>3586</v>
       </c>
       <c r="P325" t="s">
-        <v>3586</v>
+        <v>3587</v>
       </c>
       <c r="Q325" t="s">
         <v>53</v>
@@ -32508,7 +32509,7 @@
         <v>20257663</v>
       </c>
       <c r="B326" t="s">
-        <v>3587</v>
+        <v>3588</v>
       </c>
       <c r="C326" t="s">
         <v>59</v>
@@ -32520,7 +32521,7 @@
         <v>61</v>
       </c>
       <c r="F326" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G326" t="s">
         <v>27</v>
@@ -32529,26 +32530,26 @@
         <v>44</v>
       </c>
       <c r="I326" t="s">
-        <v>3588</v>
+        <v>3589</v>
       </c>
       <c r="J326" t="s">
-        <v>3589</v>
+        <v>3590</v>
       </c>
       <c r="K326"/>
       <c r="L326" t="s">
-        <v>3590</v>
+        <v>3591</v>
       </c>
       <c r="M326" t="s">
-        <v>3591</v>
+        <v>3592</v>
       </c>
       <c r="N326" t="s">
         <v>69</v>
       </c>
       <c r="O326" t="s">
-        <v>3592</v>
+        <v>3593</v>
       </c>
       <c r="P326" t="s">
-        <v>3593</v>
+        <v>3594</v>
       </c>
       <c r="Q326" t="s">
         <v>53</v>
@@ -32556,13 +32557,13 @@
       <c r="R326"/>
       <c r="S326"/>
       <c r="T326" t="s">
-        <v>3594</v>
+        <v>3595</v>
       </c>
       <c r="U326" t="s">
-        <v>3595</v>
+        <v>3596</v>
       </c>
       <c r="V326" t="s">
-        <v>3596</v>
+        <v>3597</v>
       </c>
     </row>
     <row r="327">
@@ -32570,19 +32571,19 @@
         <v>20257698</v>
       </c>
       <c r="B327" t="s">
-        <v>3597</v>
+        <v>3598</v>
       </c>
       <c r="C327" t="s">
         <v>59</v>
       </c>
       <c r="D327" t="s">
-        <v>3598</v>
+        <v>3599</v>
       </c>
       <c r="E327" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F327" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G327" t="s">
         <v>27</v>
@@ -32591,26 +32592,26 @@
         <v>44</v>
       </c>
       <c r="I327" t="s">
-        <v>3599</v>
+        <v>3600</v>
       </c>
       <c r="J327" t="s">
-        <v>3600</v>
+        <v>3601</v>
       </c>
       <c r="K327"/>
       <c r="L327" t="s">
-        <v>3601</v>
+        <v>3602</v>
       </c>
       <c r="M327" t="s">
-        <v>3602</v>
+        <v>3603</v>
       </c>
       <c r="N327" t="s">
         <v>69</v>
       </c>
       <c r="O327" t="s">
-        <v>3603</v>
+        <v>3604</v>
       </c>
       <c r="P327" t="s">
-        <v>3604</v>
+        <v>3605</v>
       </c>
       <c r="Q327" t="s">
         <v>53</v>
@@ -32632,19 +32633,19 @@
         <v>20253971</v>
       </c>
       <c r="B328" t="s">
-        <v>3605</v>
+        <v>3606</v>
       </c>
       <c r="C328" t="s">
         <v>40</v>
       </c>
       <c r="D328" t="s">
-        <v>3606</v>
+        <v>3607</v>
       </c>
       <c r="E328" t="s">
         <v>42</v>
       </c>
       <c r="F328" t="s">
-        <v>3607</v>
+        <v>3608</v>
       </c>
       <c r="G328" t="s">
         <v>81</v>
@@ -32653,28 +32654,28 @@
         <v>563</v>
       </c>
       <c r="I328" t="s">
-        <v>3608</v>
+        <v>3609</v>
       </c>
       <c r="J328" t="s">
-        <v>3609</v>
+        <v>3610</v>
       </c>
       <c r="K328" t="s">
-        <v>3610</v>
+        <v>3611</v>
       </c>
       <c r="L328" t="s">
-        <v>3611</v>
+        <v>3612</v>
       </c>
       <c r="M328" t="s">
-        <v>3612</v>
+        <v>3613</v>
       </c>
       <c r="N328" t="s">
         <v>69</v>
       </c>
       <c r="O328" t="s">
-        <v>3613</v>
+        <v>3614</v>
       </c>
       <c r="P328" t="s">
-        <v>3614</v>
+        <v>3615</v>
       </c>
       <c r="Q328" t="s">
         <v>89</v>
@@ -32682,13 +32683,13 @@
       <c r="R328"/>
       <c r="S328"/>
       <c r="T328" t="s">
-        <v>3480</v>
+        <v>3481</v>
       </c>
       <c r="U328" t="s">
-        <v>3481</v>
+        <v>3482</v>
       </c>
       <c r="V328" t="s">
-        <v>3482</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="329">
@@ -32696,7 +32697,7 @@
         <v>20257601</v>
       </c>
       <c r="B329" t="s">
-        <v>3615</v>
+        <v>3616</v>
       </c>
       <c r="C329" t="s">
         <v>59</v>
@@ -32705,10 +32706,10 @@
         <v>1495</v>
       </c>
       <c r="E329" t="s">
-        <v>1496</v>
+        <v>659</v>
       </c>
       <c r="F329" t="s">
-        <v>3616</v>
+        <v>3617</v>
       </c>
       <c r="G329" t="s">
         <v>27</v>
@@ -32717,26 +32718,26 @@
         <v>97</v>
       </c>
       <c r="I329" t="s">
-        <v>3617</v>
+        <v>3618</v>
       </c>
       <c r="J329" t="s">
-        <v>3618</v>
+        <v>3619</v>
       </c>
       <c r="K329"/>
       <c r="L329" t="s">
-        <v>3619</v>
+        <v>3620</v>
       </c>
       <c r="M329" t="s">
-        <v>3620</v>
+        <v>3621</v>
       </c>
       <c r="N329" t="s">
         <v>69</v>
       </c>
       <c r="O329" t="s">
-        <v>3621</v>
+        <v>3622</v>
       </c>
       <c r="P329" t="s">
-        <v>3622</v>
+        <v>3623</v>
       </c>
       <c r="Q329" t="s">
         <v>89</v>
@@ -32758,17 +32759,17 @@
         <v>20253941</v>
       </c>
       <c r="B330" t="s">
-        <v>3623</v>
+        <v>3624</v>
       </c>
       <c r="C330" t="s">
         <v>77</v>
       </c>
       <c r="D330" t="s">
-        <v>3624</v>
+        <v>3625</v>
       </c>
       <c r="E330"/>
       <c r="F330" t="s">
-        <v>3625</v>
+        <v>3626</v>
       </c>
       <c r="G330" t="s">
         <v>27</v>
@@ -32777,28 +32778,28 @@
         <v>1556</v>
       </c>
       <c r="I330" t="s">
-        <v>3626</v>
+        <v>3627</v>
       </c>
       <c r="J330" t="s">
-        <v>3627</v>
+        <v>3628</v>
       </c>
       <c r="K330" t="s">
-        <v>3628</v>
+        <v>3629</v>
       </c>
       <c r="L330" t="s">
-        <v>3629</v>
+        <v>3630</v>
       </c>
       <c r="M330" t="s">
-        <v>3630</v>
+        <v>3631</v>
       </c>
       <c r="N330" t="s">
         <v>1987</v>
       </c>
       <c r="O330" t="s">
-        <v>3631</v>
+        <v>3632</v>
       </c>
       <c r="P330" t="s">
-        <v>3632</v>
+        <v>3633</v>
       </c>
       <c r="Q330" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-07
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -10404,12 +10404,33 @@
     <t xml:space="preserve">Ambiente|Agricoltura</t>
   </si>
   <si>
+    <t xml:space="preserve">25.7863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Débâcle fiscale vaudoise. Conséquences sur la péréquation financière ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Des rapports datant du printemps critiquent le calcul erroné de l’impôt sur la fortune dans le canton de Vaud qui a engendré une perte pouvant se chiffrer en millions de francs. Le canton de Vaud bénéficiant de la péréquation financière nationale, les erreurs pourraient avoir des répercussions sur les autres cantons et la Confédération.&lt;br&gt;- Est-ce que le Conseil fédéral partage cette analyse&amp;nbsp;?&lt;br&gt;- Les paiements compensatoires déjà effectués peuvent-ils être corrigés&amp;nbsp;?&lt;br&gt;- Quelles mesures entend prendre le Conseil fédéral pour éviter, à l’avenir, de telles erreurs&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Berichte aus dem Frühjahr kritisieren die fehlerhafte Vermögenssteuerberechnung im Kanton Waadt, die ihm mutmasslich mehrere Millionen Franken kostete. Da Waadt Nehmerkanton im nationalen Finanzausgleich ist, könnten die Fehler auch andere Kantone und den Bund betreffen.&lt;br&gt;- Teilt der Bundesrat diese Einschätzung?&lt;br&gt;- Können bereits geleistete Ausgleichszahlungen korrigiert werden?&lt;br&gt;- Welche Massnahmen plant er, um solche Fehler künftig zu verhindern?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.4024</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
   </si>
   <si>
@@ -10431,27 +10452,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
   </si>
   <si>
-    <t xml:space="preserve">25.7863</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Débâcle fiscale vaudoise. Conséquences sur la péréquation financière ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Des rapports datant du printemps critiquent le calcul erroné de l’impôt sur la fortune dans le canton de Vaud qui a engendré une perte pouvant se chiffrer en millions de francs. Le canton de Vaud bénéficiant de la péréquation financière nationale, les erreurs pourraient avoir des répercussions sur les autres cantons et la Confédération.&lt;br&gt;- Est-ce que le Conseil fédéral partage cette analyse&amp;nbsp;?&lt;br&gt;- Les paiements compensatoires déjà effectués peuvent-ils être corrigés&amp;nbsp;?&lt;br&gt;- Quelles mesures entend prendre le Conseil fédéral pour éviter, à l’avenir, de telles erreurs&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Berichte aus dem Frühjahr kritisieren die fehlerhafte Vermögenssteuerberechnung im Kanton Waadt, die ihm mutmasslich mehrere Millionen Franken kostete. Da Waadt Nehmerkanton im nationalen Finanzausgleich ist, könnten die Fehler auch andere Kantone und den Bund betreffen.&lt;br&gt;- Teilt der Bundesrat diese Einschätzung?&lt;br&gt;- Können bereits geleistete Ausgleichszahlungen korrigiert werden?&lt;br&gt;- Welche Massnahmen plant er, um solche Fehler künftig zu verhindern?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.7888</t>
   </si>
   <si>
@@ -10533,12 +10533,66 @@
     <t xml:space="preserve">Economia|Imposte</t>
   </si>
   <si>
+    <t xml:space="preserve">25.7663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUAG : des millions pour des avocats au lieu de munition pour notre armée ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;RUAG, entre autres en lien avec certaines irrégularités, aurait engagé plus de 10 millions de francs en frais d'avocats &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html.&lt;/a&gt;&lt;br&gt;- Le Conseil fédéral tolère-t-il cette manière de sous-traiter à grands frais des tâches de gouvernance d'entreprise ?&lt;br&gt;- Entend-il prendre des mesures ?&lt;br&gt;- Ces honoraires faramineux ne seraient-ils pas mieux investis dans l'acquisition de munition ?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Die Ruag soll unter anderem im Zusammenhang mit bestimmten Unregelmässigkeiten mehr als 10 Millionen Franken für Anwaltskosten ausgegeben haben &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;(https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html).&lt;/a&gt;&lt;br&gt;– Duldet der Bundesrat diese Art der kostspieligen Auslagerung von Aufgaben der Corporate Governance?&lt;br&gt;– Beabsichtigt der Bundesrat, Massnahmen zu ergreifen?&lt;br&gt;– Wäre es nicht besser, diese enormen Beträge in den Kauf von Munition zu investieren?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sicherheitspolitik|Finanzwesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique de sécurité|Finances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica di sicurezza|Finanze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.7698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De Ventura Linda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Untersuchungskosten Ruag-Skandal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coûts de l’enquête sur le scandale RUAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;D’après la presse, les coûts de l’enquête externe sur le scandale RUAG se montent aujourd’hui à plus de 10&amp;nbsp;millions de francs.&lt;br&gt;- Quel est le montant des coûts engagés jusqu’à présent et à qui cet argent a-t-il été versé&amp;nbsp;?&lt;br&gt;- Le Conseil fédéral juge-t-il ces coûts raisonnables&amp;nbsp;? Comment justifie-t-il une telle dépense&amp;nbsp;?&lt;br&gt;- Comment explique-t-il l’évidente faillite des mécanismes de contrôle internes, à la fois dans l’entreprise RUAG et au DDPS, qui a imposé cette enquête externe&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Gemäss Medienberichten belaufen sich die Kosten für die externe Untersuchung des RUAG-Skandals inzwischen auf über CHF 10 Millionen.&lt;br&gt;- Wie hoch sind die bisherigen Kosten der Untersuchung und an wen wurden diese Mittel ausbezahlt?&lt;br&gt;- Hält der Bundesrat diese Kosten für verhältnismässig und wie rechtfertigt er sie?&lt;br&gt;- Wie erklärt der Bundesrat das offensichtliche Versagen der internen Kontrollmechanismen innerhalb der RUAG sowie im VBS, das dazu führte, dass diese externe Untersuchung notwendig&amp;nbsp;wurde?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.3984</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-10</t>
-  </si>
-  <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
   </si>
   <si>
@@ -10549,60 +10603,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.7663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUAG : des millions pour des avocats au lieu de munition pour notre armée ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;RUAG, entre autres en lien avec certaines irrégularités, aurait engagé plus de 10 millions de francs en frais d'avocats &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html.&lt;/a&gt;&lt;br&gt;- Le Conseil fédéral tolère-t-il cette manière de sous-traiter à grands frais des tâches de gouvernance d'entreprise ?&lt;br&gt;- Entend-il prendre des mesures ?&lt;br&gt;- Ces honoraires faramineux ne seraient-ils pas mieux investis dans l'acquisition de munition ?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Die Ruag soll unter anderem im Zusammenhang mit bestimmten Unregelmässigkeiten mehr als 10 Millionen Franken für Anwaltskosten ausgegeben haben &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;(https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html).&lt;/a&gt;&lt;br&gt;– Duldet der Bundesrat diese Art der kostspieligen Auslagerung von Aufgaben der Corporate Governance?&lt;br&gt;– Beabsichtigt der Bundesrat, Massnahmen zu ergreifen?&lt;br&gt;– Wäre es nicht besser, diese enormen Beträge in den Kauf von Munition zu investieren?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sicherheitspolitik|Finanzwesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique de sécurité|Finances</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica di sicurezza|Finanze</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.7698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De Ventura Linda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Untersuchungskosten Ruag-Skandal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coûts de l’enquête sur le scandale RUAG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;D’après la presse, les coûts de l’enquête externe sur le scandale RUAG se montent aujourd’hui à plus de 10&amp;nbsp;millions de francs.&lt;br&gt;- Quel est le montant des coûts engagés jusqu’à présent et à qui cet argent a-t-il été versé&amp;nbsp;?&lt;br&gt;- Le Conseil fédéral juge-t-il ces coûts raisonnables&amp;nbsp;? Comment justifie-t-il une telle dépense&amp;nbsp;?&lt;br&gt;- Comment explique-t-il l’évidente faillite des mécanismes de contrôle internes, à la fois dans l’entreprise RUAG et au DDPS, qui a imposé cette enquête externe&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Gemäss Medienberichten belaufen sich die Kosten für die externe Untersuchung des RUAG-Skandals inzwischen auf über CHF 10 Millionen.&lt;br&gt;- Wie hoch sind die bisherigen Kosten der Untersuchung und an wen wurden diese Mittel ausbezahlt?&lt;br&gt;- Hält der Bundesrat diese Kosten für verhältnismässig und wie rechtfertigt er sie?&lt;br&gt;- Wie erklärt der Bundesrat das offensichtliche Versagen der internen Kontrollmechanismen innerhalb der RUAG sowie im VBS, das dazu führte, dass diese externe Untersuchung notwendig&amp;nbsp;wurde?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
   </si>
   <si>
     <t xml:space="preserve">25.3971</t>
@@ -31446,19 +31446,19 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>20254024</v>
+        <v>20257863</v>
       </c>
       <c r="B313" t="s">
         <v>3463</v>
       </c>
       <c r="C313" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D313" t="s">
-        <v>1606</v>
+        <v>1814</v>
       </c>
       <c r="E313" t="s">
-        <v>25</v>
+        <v>1815</v>
       </c>
       <c r="F313" t="s">
         <v>3464</v>
@@ -31467,7 +31467,7 @@
         <v>27</v>
       </c>
       <c r="H313" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I313" t="s">
         <v>3465</v>
@@ -31475,54 +31475,52 @@
       <c r="J313" t="s">
         <v>3466</v>
       </c>
-      <c r="K313" t="s">
+      <c r="K313"/>
+      <c r="L313" t="s">
         <v>3467</v>
       </c>
-      <c r="L313" t="s">
+      <c r="M313" t="s">
         <v>3468</v>
       </c>
-      <c r="M313" t="s">
+      <c r="N313" t="s">
+        <v>84</v>
+      </c>
+      <c r="O313" t="s">
         <v>3469</v>
       </c>
-      <c r="N313" t="s">
-        <v>66</v>
-      </c>
-      <c r="O313" t="s">
+      <c r="P313" t="s">
         <v>3470</v>
       </c>
-      <c r="P313" t="s">
-        <v>3471</v>
-      </c>
       <c r="Q313" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="R313"/>
       <c r="S313"/>
       <c r="T313" t="s">
-        <v>1534</v>
+        <v>942</v>
       </c>
       <c r="U313" t="s">
-        <v>1535</v>
+        <v>943</v>
       </c>
       <c r="V313" t="s">
-        <v>1536</v>
+        <v>944</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>20257863</v>
+        <v>20254024</v>
       </c>
       <c r="B314" t="s">
-        <v>3472</v>
+        <v>3471</v>
       </c>
       <c r="C314" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D314" t="s">
-        <v>1814</v>
+        <v>1606</v>
       </c>
       <c r="E314" t="s">
-        <v>1815</v>
+        <v>25</v>
       </c>
       <c r="F314" t="s">
         <v>3464</v>
@@ -31531,15 +31529,17 @@
         <v>27</v>
       </c>
       <c r="H314" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I314" t="s">
+        <v>3472</v>
+      </c>
+      <c r="J314" t="s">
         <v>3473</v>
       </c>
-      <c r="J314" t="s">
+      <c r="K314" t="s">
         <v>3474</v>
       </c>
-      <c r="K314"/>
       <c r="L314" t="s">
         <v>3475</v>
       </c>
@@ -31547,7 +31547,7 @@
         <v>3476</v>
       </c>
       <c r="N314" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="O314" t="s">
         <v>3477</v>
@@ -31556,18 +31556,18 @@
         <v>3478</v>
       </c>
       <c r="Q314" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>942</v>
+        <v>1534</v>
       </c>
       <c r="U314" t="s">
-        <v>943</v>
+        <v>1535</v>
       </c>
       <c r="V314" t="s">
-        <v>944</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="315">
@@ -31758,18 +31758,20 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>20253984</v>
+        <v>20257663</v>
       </c>
       <c r="B318" t="s">
         <v>3506</v>
       </c>
       <c r="C318" t="s">
-        <v>92</v>
+        <v>23</v>
       </c>
       <c r="D318" t="s">
-        <v>623</v>
-      </c>
-      <c r="E318"/>
+        <v>163</v>
+      </c>
+      <c r="E318" t="s">
+        <v>76</v>
+      </c>
       <c r="F318" t="s">
         <v>3507</v>
       </c>
@@ -31777,31 +31779,29 @@
         <v>27</v>
       </c>
       <c r="H318" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I318" t="s">
-        <v>3411</v>
+        <v>3508</v>
       </c>
       <c r="J318" t="s">
-        <v>3412</v>
-      </c>
-      <c r="K318" t="s">
-        <v>3413</v>
-      </c>
+        <v>3509</v>
+      </c>
+      <c r="K318"/>
       <c r="L318" t="s">
-        <v>3508</v>
+        <v>3510</v>
       </c>
       <c r="M318" t="s">
-        <v>3509</v>
+        <v>3511</v>
       </c>
       <c r="N318" t="s">
-        <v>3345</v>
+        <v>84</v>
       </c>
       <c r="O318" t="s">
-        <v>3510</v>
+        <v>3512</v>
       </c>
       <c r="P318" t="s">
-        <v>3511</v>
+        <v>3513</v>
       </c>
       <c r="Q318" t="s">
         <v>69</v>
@@ -31809,30 +31809,30 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>146</v>
+        <v>3514</v>
       </c>
       <c r="U318" t="s">
-        <v>147</v>
+        <v>3515</v>
       </c>
       <c r="V318" t="s">
-        <v>148</v>
+        <v>3516</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>20257663</v>
+        <v>20257698</v>
       </c>
       <c r="B319" t="s">
-        <v>3512</v>
+        <v>3517</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
       </c>
       <c r="D319" t="s">
-        <v>163</v>
+        <v>3518</v>
       </c>
       <c r="E319" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="F319" t="s">
         <v>3507</v>
@@ -31844,26 +31844,26 @@
         <v>60</v>
       </c>
       <c r="I319" t="s">
-        <v>3513</v>
+        <v>3519</v>
       </c>
       <c r="J319" t="s">
-        <v>3514</v>
+        <v>3520</v>
       </c>
       <c r="K319"/>
       <c r="L319" t="s">
-        <v>3515</v>
+        <v>3521</v>
       </c>
       <c r="M319" t="s">
-        <v>3516</v>
+        <v>3522</v>
       </c>
       <c r="N319" t="s">
         <v>84</v>
       </c>
       <c r="O319" t="s">
-        <v>3517</v>
+        <v>3523</v>
       </c>
       <c r="P319" t="s">
-        <v>3518</v>
+        <v>3524</v>
       </c>
       <c r="Q319" t="s">
         <v>69</v>
@@ -31871,31 +31871,29 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>3519</v>
+        <v>1499</v>
       </c>
       <c r="U319" t="s">
-        <v>3520</v>
+        <v>1500</v>
       </c>
       <c r="V319" t="s">
-        <v>3521</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>20257698</v>
+        <v>20253984</v>
       </c>
       <c r="B320" t="s">
-        <v>3522</v>
+        <v>3525</v>
       </c>
       <c r="C320" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D320" t="s">
-        <v>3523</v>
-      </c>
-      <c r="E320" t="s">
-        <v>25</v>
-      </c>
+        <v>623</v>
+      </c>
+      <c r="E320"/>
       <c r="F320" t="s">
         <v>3507</v>
       </c>
@@ -31903,15 +31901,17 @@
         <v>27</v>
       </c>
       <c r="H320" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I320" t="s">
-        <v>3524</v>
+        <v>3411</v>
       </c>
       <c r="J320" t="s">
-        <v>3525</v>
-      </c>
-      <c r="K320"/>
+        <v>3412</v>
+      </c>
+      <c r="K320" t="s">
+        <v>3413</v>
+      </c>
       <c r="L320" t="s">
         <v>3526</v>
       </c>
@@ -31919,7 +31919,7 @@
         <v>3527</v>
       </c>
       <c r="N320" t="s">
-        <v>84</v>
+        <v>3345</v>
       </c>
       <c r="O320" t="s">
         <v>3528</v>
@@ -31933,13 +31933,13 @@
       <c r="R320"/>
       <c r="S320"/>
       <c r="T320" t="s">
-        <v>1499</v>
+        <v>146</v>
       </c>
       <c r="U320" t="s">
-        <v>1500</v>
+        <v>147</v>
       </c>
       <c r="V320" t="s">
-        <v>1501</v>
+        <v>148</v>
       </c>
     </row>
     <row r="321">

</xml_diff>

<commit_message>
Update parliament data - 2026-03-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -10404,12 +10404,36 @@
     <t xml:space="preserve">Ambiente|Agricoltura</t>
   </si>
   <si>
+    <t xml:space="preserve">25.4024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le DDPS confie de grands projets à des externes. Quel est l'objectif stratégique ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progetti di grande portata nel DDPS a fornitori di prestazioni esterni. Quale strategia viene seguita?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Pourquoi le DDPS externalise-t-il intégralement la gestion des risques et de la qualité de ses grands projets au lieu de renforcer des services internes tels que le Contrôle fédéral des finances ou la révision interne&amp;nbsp;?&lt;/p&gt;&lt;p&gt;2. À combien sont estimés les coûts des nouveaux contrats-cadres conclus pour une durée de douze ans&amp;nbsp;? Comment s’assure-t-on que les coûts ne dérapent pas&amp;nbsp;?&lt;/p&gt;&lt;p&gt;3. Pourquoi avoir choisi une durée de contrat aussi longue&amp;nbsp;? Est-il possible de modifier ou de résilier les contrats en cas de besoin&amp;nbsp;?&lt;/p&gt;&lt;p&gt;4. Quels critères ont déterminé le choix des prestataires externes&amp;nbsp;? Comment éviter les conflits d’intérêts et garantir l’indépendance&amp;nbsp;?&lt;/p&gt;&lt;p&gt;5. Quelles leçons le DDPS tire-t-il de précédentes expertises réalisées par des externes comme celle du cabinet d’avocat Homburger sur le F-35, qui a été taxée d’être un rapport de complaisance&amp;nbsp;? Comment la transparence sera-t-il garantie&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Weshalb lagert das VBS das Qualitäts- und Risikomanagement bei seinen Grossprojekten vollständig an Externe aus, anstatt interne Stellen wie die EFK oder die interne Revision zu stärken?&lt;/p&gt;&lt;p&gt;2. Wie hoch werden die Kosten der neuen Rahmenverträge über zwölf Jahre geschätzt, und wie wird sichergestellt, dass diese nicht aus dem Ruder laufen?&lt;/p&gt;&lt;p&gt;3. Weshalb wurde eine so lange Vertragsdauer gewählt, und welche Möglichkeiten bestehen, Verträge bei Bedarf anzupassen oder zu beenden?&lt;/p&gt;&lt;p&gt;4. Nach welchen Kriterien werden die externen Dienstleister ausgewählt, und wie wird verhindert, dass Interessenkonflikte entstehen oder die Unabhängigkeit beeinträchtigt wird?&lt;/p&gt;&lt;p&gt;5. Welche Lehren zieht das VBS aus früheren externen Gutachten wie jenen der Kanzlei Homburger zum F-35, die als Gefälligkeitsgutachten kritisiert wurden, und wie wird künftig Transparenz garantiert?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.7863</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
   </si>
   <si>
@@ -10428,30 +10452,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
   </si>
   <si>
-    <t xml:space="preserve">25.4024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le DDPS confie de grands projets à des externes. Quel est l'objectif stratégique ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progetti di grande portata nel DDPS a fornitori di prestazioni esterni. Quale strategia viene seguita?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Pourquoi le DDPS externalise-t-il intégralement la gestion des risques et de la qualité de ses grands projets au lieu de renforcer des services internes tels que le Contrôle fédéral des finances ou la révision interne&amp;nbsp;?&lt;/p&gt;&lt;p&gt;2. À combien sont estimés les coûts des nouveaux contrats-cadres conclus pour une durée de douze ans&amp;nbsp;? Comment s’assure-t-on que les coûts ne dérapent pas&amp;nbsp;?&lt;/p&gt;&lt;p&gt;3. Pourquoi avoir choisi une durée de contrat aussi longue&amp;nbsp;? Est-il possible de modifier ou de résilier les contrats en cas de besoin&amp;nbsp;?&lt;/p&gt;&lt;p&gt;4. Quels critères ont déterminé le choix des prestataires externes&amp;nbsp;? Comment éviter les conflits d’intérêts et garantir l’indépendance&amp;nbsp;?&lt;/p&gt;&lt;p&gt;5. Quelles leçons le DDPS tire-t-il de précédentes expertises réalisées par des externes comme celle du cabinet d’avocat Homburger sur le F-35, qui a été taxée d’être un rapport de complaisance&amp;nbsp;? Comment la transparence sera-t-il garantie&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Weshalb lagert das VBS das Qualitäts- und Risikomanagement bei seinen Grossprojekten vollständig an Externe aus, anstatt interne Stellen wie die EFK oder die interne Revision zu stärken?&lt;/p&gt;&lt;p&gt;2. Wie hoch werden die Kosten der neuen Rahmenverträge über zwölf Jahre geschätzt, und wie wird sichergestellt, dass diese nicht aus dem Ruder laufen?&lt;/p&gt;&lt;p&gt;3. Weshalb wurde eine so lange Vertragsdauer gewählt, und welche Möglichkeiten bestehen, Verträge bei Bedarf anzupassen oder zu beenden?&lt;/p&gt;&lt;p&gt;4. Nach welchen Kriterien werden die externen Dienstleister ausgewählt, und wie wird verhindert, dass Interessenkonflikte entstehen oder die Unabhängigkeit beeinträchtigt wird?&lt;/p&gt;&lt;p&gt;5. Welche Lehren zieht das VBS aus früheren externen Gutachten wie jenen der Kanzlei Homburger zum F-35, die als Gefälligkeitsgutachten kritisiert wurden, und wie wird künftig Transparenz garantiert?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.7888</t>
   </si>
   <si>
@@ -10533,12 +10533,27 @@
     <t xml:space="preserve">Economia|Imposte</t>
   </si>
   <si>
+    <t xml:space="preserve">25.3984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Subventionsprüfung gemäss Subventionsgesetz (SuG) so anzupassen, dass daraus ein Paket für einen Abbau von schädlichen Subventionen hervorgeht.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.7663</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
   </si>
   <si>
@@ -10588,21 +10603,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.3984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Subventionsprüfung gemäss Subventionsgesetz (SuG) so anzupassen, dass daraus ein Paket für einen Abbau von schädlichen Subventionen hervorgeht.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
   </si>
   <si>
     <t xml:space="preserve">25.3971</t>
@@ -31446,19 +31446,19 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>20257863</v>
+        <v>20254024</v>
       </c>
       <c r="B313" t="s">
         <v>3463</v>
       </c>
       <c r="C313" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D313" t="s">
-        <v>1814</v>
+        <v>1606</v>
       </c>
       <c r="E313" t="s">
-        <v>1815</v>
+        <v>25</v>
       </c>
       <c r="F313" t="s">
         <v>3464</v>
@@ -31467,7 +31467,7 @@
         <v>27</v>
       </c>
       <c r="H313" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I313" t="s">
         <v>3465</v>
@@ -31475,52 +31475,54 @@
       <c r="J313" t="s">
         <v>3466</v>
       </c>
-      <c r="K313"/>
+      <c r="K313" t="s">
+        <v>3467</v>
+      </c>
       <c r="L313" t="s">
-        <v>3467</v>
+        <v>3468</v>
       </c>
       <c r="M313" t="s">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="N313" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="O313" t="s">
-        <v>3469</v>
+        <v>3470</v>
       </c>
       <c r="P313" t="s">
-        <v>3470</v>
+        <v>3471</v>
       </c>
       <c r="Q313" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="R313"/>
       <c r="S313"/>
       <c r="T313" t="s">
-        <v>942</v>
+        <v>1534</v>
       </c>
       <c r="U313" t="s">
-        <v>943</v>
+        <v>1535</v>
       </c>
       <c r="V313" t="s">
-        <v>944</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>20254024</v>
+        <v>20257863</v>
       </c>
       <c r="B314" t="s">
-        <v>3471</v>
+        <v>3472</v>
       </c>
       <c r="C314" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D314" t="s">
-        <v>1606</v>
+        <v>1814</v>
       </c>
       <c r="E314" t="s">
-        <v>25</v>
+        <v>1815</v>
       </c>
       <c r="F314" t="s">
         <v>3464</v>
@@ -31529,17 +31531,15 @@
         <v>27</v>
       </c>
       <c r="H314" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I314" t="s">
-        <v>3472</v>
+        <v>3473</v>
       </c>
       <c r="J314" t="s">
-        <v>3473</v>
-      </c>
-      <c r="K314" t="s">
         <v>3474</v>
       </c>
+      <c r="K314"/>
       <c r="L314" t="s">
         <v>3475</v>
       </c>
@@ -31547,7 +31547,7 @@
         <v>3476</v>
       </c>
       <c r="N314" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="O314" t="s">
         <v>3477</v>
@@ -31556,18 +31556,18 @@
         <v>3478</v>
       </c>
       <c r="Q314" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>1534</v>
+        <v>942</v>
       </c>
       <c r="U314" t="s">
-        <v>1535</v>
+        <v>943</v>
       </c>
       <c r="V314" t="s">
-        <v>1536</v>
+        <v>944</v>
       </c>
     </row>
     <row r="315">
@@ -31758,20 +31758,18 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>20257663</v>
+        <v>20253984</v>
       </c>
       <c r="B318" t="s">
         <v>3506</v>
       </c>
       <c r="C318" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D318" t="s">
-        <v>163</v>
-      </c>
-      <c r="E318" t="s">
-        <v>76</v>
-      </c>
+        <v>623</v>
+      </c>
+      <c r="E318"/>
       <c r="F318" t="s">
         <v>3507</v>
       </c>
@@ -31779,29 +31777,31 @@
         <v>27</v>
       </c>
       <c r="H318" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I318" t="s">
+        <v>3411</v>
+      </c>
+      <c r="J318" t="s">
+        <v>3412</v>
+      </c>
+      <c r="K318" t="s">
+        <v>3413</v>
+      </c>
+      <c r="L318" t="s">
         <v>3508</v>
       </c>
-      <c r="J318" t="s">
+      <c r="M318" t="s">
         <v>3509</v>
       </c>
-      <c r="K318"/>
-      <c r="L318" t="s">
+      <c r="N318" t="s">
+        <v>3345</v>
+      </c>
+      <c r="O318" t="s">
         <v>3510</v>
       </c>
-      <c r="M318" t="s">
+      <c r="P318" t="s">
         <v>3511</v>
-      </c>
-      <c r="N318" t="s">
-        <v>84</v>
-      </c>
-      <c r="O318" t="s">
-        <v>3512</v>
-      </c>
-      <c r="P318" t="s">
-        <v>3513</v>
       </c>
       <c r="Q318" t="s">
         <v>69</v>
@@ -31809,30 +31809,30 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>3514</v>
+        <v>146</v>
       </c>
       <c r="U318" t="s">
-        <v>3515</v>
+        <v>147</v>
       </c>
       <c r="V318" t="s">
-        <v>3516</v>
+        <v>148</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>20257698</v>
+        <v>20257663</v>
       </c>
       <c r="B319" t="s">
-        <v>3517</v>
+        <v>3512</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
       </c>
       <c r="D319" t="s">
-        <v>3518</v>
+        <v>163</v>
       </c>
       <c r="E319" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="F319" t="s">
         <v>3507</v>
@@ -31844,26 +31844,26 @@
         <v>60</v>
       </c>
       <c r="I319" t="s">
-        <v>3519</v>
+        <v>3513</v>
       </c>
       <c r="J319" t="s">
-        <v>3520</v>
+        <v>3514</v>
       </c>
       <c r="K319"/>
       <c r="L319" t="s">
-        <v>3521</v>
+        <v>3515</v>
       </c>
       <c r="M319" t="s">
-        <v>3522</v>
+        <v>3516</v>
       </c>
       <c r="N319" t="s">
         <v>84</v>
       </c>
       <c r="O319" t="s">
-        <v>3523</v>
+        <v>3517</v>
       </c>
       <c r="P319" t="s">
-        <v>3524</v>
+        <v>3518</v>
       </c>
       <c r="Q319" t="s">
         <v>69</v>
@@ -31871,29 +31871,31 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>1499</v>
+        <v>3519</v>
       </c>
       <c r="U319" t="s">
-        <v>1500</v>
+        <v>3520</v>
       </c>
       <c r="V319" t="s">
-        <v>1501</v>
+        <v>3521</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>20253984</v>
+        <v>20257698</v>
       </c>
       <c r="B320" t="s">
-        <v>3525</v>
+        <v>3522</v>
       </c>
       <c r="C320" t="s">
-        <v>92</v>
+        <v>23</v>
       </c>
       <c r="D320" t="s">
-        <v>623</v>
-      </c>
-      <c r="E320"/>
+        <v>3523</v>
+      </c>
+      <c r="E320" t="s">
+        <v>25</v>
+      </c>
       <c r="F320" t="s">
         <v>3507</v>
       </c>
@@ -31901,17 +31903,15 @@
         <v>27</v>
       </c>
       <c r="H320" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I320" t="s">
-        <v>3411</v>
+        <v>3524</v>
       </c>
       <c r="J320" t="s">
-        <v>3412</v>
-      </c>
-      <c r="K320" t="s">
-        <v>3413</v>
-      </c>
+        <v>3525</v>
+      </c>
+      <c r="K320"/>
       <c r="L320" t="s">
         <v>3526</v>
       </c>
@@ -31919,7 +31919,7 @@
         <v>3527</v>
       </c>
       <c r="N320" t="s">
-        <v>3345</v>
+        <v>84</v>
       </c>
       <c r="O320" t="s">
         <v>3528</v>
@@ -31933,13 +31933,13 @@
       <c r="R320"/>
       <c r="S320"/>
       <c r="T320" t="s">
-        <v>146</v>
+        <v>1499</v>
       </c>
       <c r="U320" t="s">
-        <v>147</v>
+        <v>1500</v>
       </c>
       <c r="V320" t="s">
-        <v>148</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="321">

</xml_diff>